<commit_message>
Perbaiki rumus rekap kuesioner (nama sheet ikut terganti)
</commit_message>
<xml_diff>
--- a/docs/rekap-kuesioner.xlsx
+++ b/docs/rekap-kuesioner.xlsx
@@ -492,451 +492,151 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -992,7 +692,6 @@
         <f>AVERAGE(Data!D2:D31)</f>
         <v/>
       </c>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1004,10 +703,9 @@
         </is>
       </c>
       <c r="C3">
-        <f>AVERAGE(Eata!E2:E31)</f>
-        <v/>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <f>AVERAGE(Data!E2:E31)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1019,10 +717,9 @@
         </is>
       </c>
       <c r="C4">
-        <f>AVERAGE(Fata!F2:F31)</f>
-        <v/>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <f>AVERAGE(Data!F2:F31)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1034,10 +731,9 @@
         </is>
       </c>
       <c r="C5">
-        <f>AVERAGE(Gata!G2:G31)</f>
-        <v/>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <f>AVERAGE(Data!G2:G31)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1049,10 +745,9 @@
         </is>
       </c>
       <c r="C6">
-        <f>AVERAGE(Hata!H2:H31)</f>
-        <v/>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <f>AVERAGE(Data!H2:H31)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1064,10 +759,9 @@
         </is>
       </c>
       <c r="C7">
-        <f>AVERAGE(Iata!I2:I31)</f>
-        <v/>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <f>AVERAGE(Data!I2:I31)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1079,10 +773,9 @@
         </is>
       </c>
       <c r="C8">
-        <f>AVERAGE(Jata!J2:J31)</f>
-        <v/>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <f>AVERAGE(Data!J2:J31)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1094,10 +787,9 @@
         </is>
       </c>
       <c r="C9">
-        <f>AVERAGE(Kata!K2:K31)</f>
-        <v/>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <f>AVERAGE(Data!K2:K31)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1105,12 +797,10 @@
           <t>Rata-rata keseluruhan</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11">
         <f>AVERAGE(C2:C9)</f>
         <v/>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1118,12 +808,10 @@
           <t>Jumlah responden</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12">
         <f>COUNTA(Data!A2:A31)</f>
         <v/>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1131,9 +819,6 @@
           <t>Panduan interpretasi:</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1146,8 +831,6 @@
           <t>Sangat Baik</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1160,8 +843,6 @@
           <t>Baik</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1174,8 +855,6 @@
           <t>Cukup</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1188,8 +867,6 @@
           <t>Kurang</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1202,8 +879,6 @@
           <t>Sangat Kurang</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>